<commit_message>
feat: cadastro de produtos B2B — SKU, variações e importação inteligente
- Adiciona campos sku, description, has_variants, base_unit na tabela products
- Cria tabela product_variants com peso, gramatura, dimensões, cor, tamanho e custom_attributes
- Funções SQL para geração automática de SKU (formato TIPO-0001)
- Migration gera SKU para produtos existentes
- Hook useProductVariants com CRUD completo + bulk create
- Hook useProductsWithVariants para buscar produtos com variações
- CreateProductModal e EditProductModal com seção de variações inline
- ProductImportModal refatorado: mapeamento flexível de colunas, suporte a variações via parent_sku, atualização em massa por SKU
- Página Produtos exibe SKU, badge de variações e faixa de preço
- Template de importação atualizado com exemplos de produtos e variações

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/products_import_template.xlsx
+++ b/public/products_import_template.xlsx
@@ -397,81 +397,529 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:T8"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>sku</v>
+      </c>
+      <c r="B1" t="str">
+        <v>parent_sku</v>
+      </c>
+      <c r="C1" t="str">
         <v>name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
         <v>type</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
+        <v>description</v>
+      </c>
+      <c r="F1" t="str">
+        <v>base_unit</v>
+      </c>
+      <c r="G1" t="str">
         <v>ticket</v>
       </c>
-      <c r="D1" t="str">
+      <c r="H1" t="str">
         <v>ticket_minimo</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
         <v>entregaveis</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>materiais</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>links</v>
       </c>
-      <c r="H1" t="str">
+      <c r="L1" t="str">
         <v>logo_url</v>
       </c>
-      <c r="I1" t="str">
+      <c r="M1" t="str">
         <v>contrato_padrao_url</v>
       </c>
-      <c r="J1" t="str">
+      <c r="N1" t="str">
         <v>contrato_minimo_url</v>
       </c>
-      <c r="K1" t="str">
+      <c r="O1" t="str">
+        <v>weight</v>
+      </c>
+      <c r="P1" t="str">
+        <v>grammage</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>dimensions</v>
+      </c>
+      <c r="R1" t="str">
+        <v>color</v>
+      </c>
+      <c r="S1" t="str">
+        <v>size</v>
+      </c>
+      <c r="T1" t="str">
         <v>is_active</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Exemplo MRR</v>
+        <v>MRR-0001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>Software CRM</v>
+      </c>
+      <c r="D2" t="str">
         <v>mrr</v>
       </c>
-      <c r="C2">
+      <c r="E2" t="str">
+        <v>Sistema de gestão de clientes</v>
+      </c>
+      <c r="F2" t="str">
+        <v>licença</v>
+      </c>
+      <c r="G2">
+        <v>200</v>
+      </c>
+      <c r="H2">
         <v>100</v>
       </c>
-      <c r="D2">
-        <v>50</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Descrição dos entregáveis</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Materiais de apoio</v>
-      </c>
-      <c r="G2" t="str">
-        <v>https://exemplo.com;https://outro.com</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Acesso ao sistema + suporte</v>
       </c>
       <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
+        <v>Manual do usuário</v>
+      </c>
+      <c r="K2" t="str">
+        <v>https://exemplo.com;https://docs.exemplo.com</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PRJ-0001</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Consultoria Empresarial</v>
+      </c>
+      <c r="D3" t="str">
+        <v>projeto</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Pacote de consultoria personalizada</v>
+      </c>
+      <c r="F3" t="str">
+        <v>hora</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>Relatório final + plano de ação</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PRJ-0001-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PRJ-0001</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Pacote Básico (10h)</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>5000</v>
+      </c>
+      <c r="H4">
+        <v>3000</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PRJ-0001-02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PRJ-0001</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pacote Premium (40h)</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>18000</v>
+      </c>
+      <c r="H5">
+        <v>12000</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>UNI-0001</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v>Material Impresso</v>
+      </c>
+      <c r="D6" t="str">
+        <v>unitario</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Material impresso personalizado</v>
+      </c>
+      <c r="F6" t="str">
+        <v>unidade</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Impressão + acabamento</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>UNI-0001-01</v>
+      </c>
+      <c r="B7" t="str">
+        <v>UNI-0001</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Flyer A5 - 150g</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7">
+        <v>2.5</v>
+      </c>
+      <c r="H7">
+        <v>1.5</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7">
+        <v>0.01</v>
+      </c>
+      <c r="P7">
+        <v>150</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>21x14.8 cm</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v>A5</v>
+      </c>
+      <c r="T7" t="str">
+        <v>sim</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>UNI-0001-02</v>
+      </c>
+      <c r="B8" t="str">
+        <v>UNI-0001</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Flyer A4 - 300g</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8">
+        <v>0.02</v>
+      </c>
+      <c r="P8">
+        <v>300</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>29.7x21 cm</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v>A4</v>
+      </c>
+      <c r="T8" t="str">
+        <v>sim</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>